<commit_message>
Improve region matching for new bids by using additional company information
Add `gcOfficeHint` field to `BcOpportunity` interface and update `mapOpportunityToEntry` to use it as a fallback for region matching, along with a new `extractOfficeCity` helper function.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0b85d283-1a28-4a74-80f4-65cba99254bc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/O80y0qk
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-02.xlsx
+++ b/backups/proposal-log-2026-04-02.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="56">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -155,6 +155,30 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
+  </si>
+  <si>
+    <t>26-0204</t>
+  </si>
+  <si>
+    <t>TRA General Office Complex</t>
+  </si>
+  <si>
+    <t>Office</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>Christman Weeks</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69ce6ad9ffa00f5f6b96a4d9</t>
   </si>
 </sst>
 </file>
@@ -553,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -789,8 +813,52 @@
         <v>47</v>
       </c>
     </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>54</v>
+      </c>
+      <c r="K6" t="s">
+        <v>17</v>
+      </c>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N5"/>
+  <autoFilter ref="A1:N6"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve region matching for project proposals by prioritizing office hints
Update region matching logic to prioritize office hints and add "parking structures" to TM region aliases.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f727589a-eb4c-4666-bc9e-2f8a4c1767dc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/QE9eINt
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-02.xlsx
+++ b/backups/proposal-log-2026-04-02.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -137,48 +137,6 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69bc538e7aaadb003896155f</t>
-  </si>
-  <si>
-    <t>Amazon SEA Legacy Space Refresh Medium GC Bid</t>
-  </si>
-  <si>
-    <t>ATL - Atlanta</t>
-  </si>
-  <si>
-    <t>2026-04-09</t>
-  </si>
-  <si>
-    <t>HK</t>
-  </si>
-  <si>
-    <t>Merci Keathley</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
-  </si>
-  <si>
-    <t>26-0204</t>
-  </si>
-  <si>
-    <t>TRA General Office Complex</t>
-  </si>
-  <si>
-    <t>Office</t>
-  </si>
-  <si>
-    <t>2026-04-02</t>
-  </si>
-  <si>
-    <t>2026-04-23</t>
-  </si>
-  <si>
-    <t>Christman Weeks</t>
-  </si>
-  <si>
-    <t>Draft</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69ce6ad9ffa00f5f6b96a4d9</t>
   </si>
 </sst>
 </file>
@@ -577,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -769,96 +727,8 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" t="s">
-        <v>46</v>
-      </c>
-      <c r="I5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" t="s">
-        <v>17</v>
-      </c>
-      <c r="L5" t="s">
-        <v>17</v>
-      </c>
-      <c r="M5" t="s">
-        <v>17</v>
-      </c>
-      <c r="N5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>53</v>
-      </c>
-      <c r="I6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" t="s">
-        <v>54</v>
-      </c>
-      <c r="K6" t="s">
-        <v>17</v>
-      </c>
-      <c r="L6" t="s">
-        <v>17</v>
-      </c>
-      <c r="M6" t="s">
-        <v>17</v>
-      </c>
-      <c r="N6" t="s">
-        <v>55</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:N4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>